<commit_message>
prvi scenario - koraci 8,9,10
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="10188"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
   <si>
     <t>username</t>
   </si>
@@ -96,6 +96,15 @@
   </si>
   <si>
     <t>REN 021</t>
+  </si>
+  <si>
+    <t>SUR ŠKOLARAC</t>
+  </si>
+  <si>
+    <t>PROCODEX</t>
+  </si>
+  <si>
+    <t>ŠIFO</t>
   </si>
 </sst>
 </file>
@@ -108,7 +117,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,16 +134,12 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10.5"/>
-      <color theme="1"/>
-      <name val="Segoe UI"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -596,134 +601,134 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -733,16 +738,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1064,8 +1069,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M11"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6"/>
   <cols>
     <col min="1" max="1" width="37.2222222222222" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.712962962963" style="1" customWidth="1"/>
@@ -1080,7 +1085,7 @@
     <col min="11" max="16384" width="8.88888888888889" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:13">
+    <row r="1" s="1" customFormat="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1112,7 +1117,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:13">
+    <row r="2" s="1" customFormat="1" spans="1:10">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -1140,18 +1145,18 @@
       <c r="I2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:13">
+    <row r="3" s="1" customFormat="1" spans="1:10">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -1172,12 +1177,12 @@
       <c r="I3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" spans="1:13">
-      <c r="A4" s="2" t="s">
+    <row r="4" s="1" customFormat="1" spans="1:10">
+      <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -1204,94 +1209,60 @@
       <c r="I4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" ht="16.8" spans="1:13">
-      <c r="D5" s="3"/>
-      <c r="E5"/>
-      <c r="F5"/>
-      <c r="G5"/>
-      <c r="H5"/>
-      <c r="I5"/>
-      <c r="J5"/>
-      <c r="K5"/>
-      <c r="L5"/>
-      <c r="M5"/>
+    <row r="5" spans="1:10">
+      <c r="A5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1">
+        <v>50100796</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="1">
+        <v>113913661</v>
+      </c>
     </row>
-    <row r="6" spans="1:13">
-      <c r="D6"/>
-      <c r="E6"/>
-      <c r="F6"/>
-      <c r="G6"/>
-      <c r="H6"/>
-      <c r="I6"/>
-      <c r="J6"/>
-      <c r="K6"/>
-      <c r="L6"/>
-      <c r="M6"/>
+    <row r="6" spans="1:10">
+      <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="1">
+        <v>20024623</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="1">
+        <v>104196650</v>
+      </c>
     </row>
-    <row r="7" spans="1:13">
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-    </row>
-    <row r="8" spans="1:13">
-      <c r="D8"/>
-      <c r="E8"/>
-      <c r="F8"/>
-      <c r="G8"/>
-      <c r="H8"/>
-      <c r="I8"/>
-      <c r="J8"/>
-      <c r="K8"/>
-      <c r="L8"/>
-      <c r="M8"/>
-    </row>
-    <row r="9" ht="16.8" spans="1:13">
-      <c r="C9" s="5"/>
-      <c r="D9" s="3"/>
-      <c r="E9"/>
-      <c r="F9"/>
-      <c r="G9"/>
-      <c r="H9"/>
-      <c r="I9"/>
-      <c r="J9"/>
-      <c r="K9"/>
-      <c r="L9"/>
-      <c r="M9"/>
-    </row>
-    <row r="10" spans="1:13">
-      <c r="D10"/>
-      <c r="E10"/>
-      <c r="F10"/>
-      <c r="G10"/>
-      <c r="H10"/>
-      <c r="I10"/>
-      <c r="J10"/>
-      <c r="K10"/>
-      <c r="L10"/>
-      <c r="M10"/>
-    </row>
-    <row r="11" ht="16.8" spans="1:13">
-      <c r="D11" s="3"/>
-      <c r="E11"/>
-      <c r="F11"/>
-      <c r="G11"/>
-      <c r="H11"/>
-      <c r="I11"/>
-      <c r="J11"/>
-      <c r="K11"/>
-      <c r="L11"/>
-      <c r="M11"/>
+    <row r="7" spans="1:10">
+      <c r="A7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="1">
+        <v>101013493</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1301,6 +1272,9 @@
     <hyperlink ref="G3" r:id="rId2" display="piljarnica.ren021@gmail.com" tooltip="mailto:piljarnica.ren021@gmail.com"/>
     <hyperlink ref="A4" r:id="rId1" display="miljan.moracanin@dtc.rs" tooltip="mailto:miljan.moracanin@dtc.rs"/>
     <hyperlink ref="G4" r:id="rId2" display="piljarnica.ren021@gmail.com" tooltip="mailto:piljarnica.ren021@gmail.com"/>
+    <hyperlink ref="A5" r:id="rId1" display="miljan.moracanin@dtc.rs" tooltip="mailto:miljan.moracanin@dtc.rs"/>
+    <hyperlink ref="A6" r:id="rId1" display="miljan.moracanin@dtc.rs"/>
+    <hyperlink ref="A7" r:id="rId1" display="miljan.moracanin@dtc.rs" tooltip="mailto:miljan.moracanin@dtc.rs"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
prvi test i dalje..
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="35">
   <si>
     <t>username</t>
   </si>
@@ -59,6 +59,9 @@
     <t>company_registration_number_invalid</t>
   </si>
   <si>
+    <t>Komentar</t>
+  </si>
+  <si>
     <t>miljan.moracanin@dtc.rs</t>
   </si>
   <si>
@@ -101,10 +104,34 @@
     <t>SUR ŠKOLARAC</t>
   </si>
   <si>
+    <t>Neispravan mb</t>
+  </si>
+  <si>
     <t>PROCODEX</t>
   </si>
   <si>
+    <t>odabir jednog od vise zastupnika</t>
+  </si>
+  <si>
     <t>ŠIFO</t>
+  </si>
+  <si>
+    <t>Aktivan Back button bez obzira na odabir zastupnika</t>
+  </si>
+  <si>
+    <t>06027415</t>
+  </si>
+  <si>
+    <t>Mol komerc</t>
+  </si>
+  <si>
+    <t>Status u stecaju</t>
+  </si>
+  <si>
+    <t>TEHNOMEDIA CENTAR</t>
+  </si>
+  <si>
+    <t>Nije u SBB segmentu</t>
   </si>
 </sst>
 </file>
@@ -1069,8 +1096,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6"/>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="37.2222222222222" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.712962962963" style="1" customWidth="1"/>
@@ -1082,10 +1109,11 @@
     <col min="8" max="8" width="29" style="1" customWidth="1"/>
     <col min="9" max="9" width="28.4259259259259" style="1" customWidth="1"/>
     <col min="10" max="10" width="33.6666666666667" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.88888888888889" style="1"/>
+    <col min="11" max="11" width="47.8888888888889" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="8.88888888888889" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:10">
+    <row r="1" s="1" customFormat="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1116,152 +1144,204 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:10">
+    <row r="2" s="1" customFormat="1" spans="1:11">
       <c r="A2" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" s="1">
         <v>50003477</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" s="1">
         <v>101351695</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:10">
+    <row r="3" s="1" customFormat="1" spans="1:11">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" s="1">
         <v>101931073</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" spans="1:10">
+    <row r="4" s="1" customFormat="1" spans="1:11">
       <c r="A4" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1">
         <v>64448170</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" s="1">
         <v>109815661</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:11">
       <c r="A5" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" s="1">
         <v>50100796</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E5" s="1">
         <v>113913661</v>
       </c>
+      <c r="K5" s="1" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:11">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="1">
         <v>20024623</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E6" s="1">
         <v>104196650</v>
       </c>
+      <c r="K6" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:11">
       <c r="A7" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E7" s="1">
         <v>101013493</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="1">
+        <v>100292243</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="1">
+        <v>20168501</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="1">
+        <v>104457054</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -1275,6 +1355,8 @@
     <hyperlink ref="A5" r:id="rId1" display="miljan.moracanin@dtc.rs" tooltip="mailto:miljan.moracanin@dtc.rs"/>
     <hyperlink ref="A6" r:id="rId1" display="miljan.moracanin@dtc.rs"/>
     <hyperlink ref="A7" r:id="rId1" display="miljan.moracanin@dtc.rs" tooltip="mailto:miljan.moracanin@dtc.rs"/>
+    <hyperlink ref="A8" r:id="rId1" display="miljan.moracanin@dtc.rs" tooltip="mailto:miljan.moracanin@dtc.rs"/>
+    <hyperlink ref="A9" r:id="rId1" display="miljan.moracanin@dtc.rs"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
happy path do mejla
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="38">
   <si>
     <t>username</t>
   </si>
@@ -62,6 +62,9 @@
     <t>Komentar</t>
   </si>
   <si>
+    <t>phone</t>
+  </si>
+  <si>
     <t>miljan.moracanin@dtc.rs</t>
   </si>
   <si>
@@ -86,6 +89,9 @@
     <t>06290965</t>
   </si>
   <si>
+    <t>happy path</t>
+  </si>
+  <si>
     <t>06066909</t>
   </si>
   <si>
@@ -96,6 +102,9 @@
   </si>
   <si>
     <t>Petković</t>
+  </si>
+  <si>
+    <t>.</t>
   </si>
   <si>
     <t>REN 021</t>
@@ -1096,7 +1105,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="37.2222222222222" style="1" customWidth="1"/>
@@ -1110,10 +1119,11 @@
     <col min="9" max="9" width="28.4259259259259" style="1" customWidth="1"/>
     <col min="10" max="10" width="33.6666666666667" style="1" customWidth="1"/>
     <col min="11" max="11" width="47.8888888888889" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.88888888888889" style="1"/>
+    <col min="12" max="12" width="10.6666666666667" style="1"/>
+    <col min="13" max="16384" width="8.88888888888889" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:11">
+    <row r="1" s="1" customFormat="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1147,201 +1157,312 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:11">
+    <row r="2" s="1" customFormat="1" spans="1:12">
       <c r="A2" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" s="1">
         <v>50003477</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" s="1">
         <v>101351695</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" s="1">
+        <v>77280402</v>
       </c>
     </row>
-    <row r="3" s="1" customFormat="1" spans="1:11">
+    <row r="3" s="1" customFormat="1" spans="1:12">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E3" s="1">
         <v>101931073</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" s="1">
+        <v>77280403</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" spans="1:11">
+    <row r="4" s="1" customFormat="1" spans="1:12">
       <c r="A4" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" s="1">
         <v>64448170</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E4" s="1">
         <v>109815661</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="L4" s="1">
+        <v>77280404</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:12">
       <c r="A5" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1">
         <v>50100796</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E5" s="1">
         <v>113913661</v>
       </c>
+      <c r="F5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>25</v>
+      </c>
       <c r="K5" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
+      </c>
+      <c r="L5" s="1">
+        <v>77280405</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:12">
       <c r="A6" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6" s="1">
         <v>20024623</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E6" s="1">
         <v>104196650</v>
       </c>
+      <c r="F6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>25</v>
+      </c>
       <c r="K6" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
+      </c>
+      <c r="L6" s="1">
+        <v>77280406</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:12">
       <c r="A7" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E7" s="1">
         <v>101013493</v>
       </c>
+      <c r="F7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>25</v>
+      </c>
       <c r="K7" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="L7" s="1">
+        <v>77280407</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:12">
       <c r="A8" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E8" s="1">
         <v>100292243</v>
       </c>
+      <c r="F8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>25</v>
+      </c>
       <c r="K8" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
+      </c>
+      <c r="L8" s="1">
+        <v>77280408</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:12">
       <c r="A9" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C9" s="1">
         <v>20168501</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E9" s="1">
         <v>104457054</v>
       </c>
+      <c r="F9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>25</v>
+      </c>
       <c r="K9" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
+      </c>
+      <c r="L9" s="1">
+        <v>77280409</v>
       </c>
     </row>
   </sheetData>

</xml_diff>